<commit_message>
#7  BOM resistor update
</commit_message>
<xml_diff>
--- a/Design-Files/PowerCutMonitor-v1.1 (Contactless Version)/BOM/JLCPCB_BOM_PowerCutMonitor-v1.1.xlsx
+++ b/Design-Files/PowerCutMonitor-v1.1 (Contactless Version)/BOM/JLCPCB_BOM_PowerCutMonitor-v1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\davetetlow-PowerCutMonitor\Design-Files\PowerCutMonitor-v1.1 (Contactless Version)\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6076395-2FA1-4A00-A7CD-D7EF31A8939B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E61A0E5-EDD9-4B49-9582-7F92423A710F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="126">
   <si>
     <t>Comment</t>
   </si>
@@ -400,6 +400,15 @@
   </si>
   <si>
     <t>R13, R14</t>
+  </si>
+  <si>
+    <t>0R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R11 </t>
+  </si>
+  <si>
+    <t>C106231</t>
   </si>
 </sst>
 </file>
@@ -840,13 +849,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="19.33203125" customWidth="1"/>
-    <col min="4" max="4" width="26.5546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1073,7 +1082,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" ht="24">
       <c r="A17" s="6" t="s">
         <v>56</v>
       </c>
@@ -1283,7 +1292,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" ht="24">
       <c r="A32" s="6" t="s">
         <v>103</v>
       </c>
@@ -1337,6 +1346,20 @@
       </c>
       <c r="D35" s="4" t="s">
         <v>117</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>